<commit_message>
fix: correct Amazon MUNBYN row column shift and update TOTAL row
Row was shifted one column right — fixed to align with all other rows.
TOTAL row updated: subtotal $4,983.65, tax $279.05, grand total $5,483.07.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/receipts/American_Select_Expenses.xlsx
+++ b/receipts/American_Select_Expenses.xlsx
@@ -676,12 +676,14 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3591,7 +3593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>133</v>
       </c>
@@ -3623,35 +3625,35 @@
         <v>56</v>
       </c>
     </row>
-    <row r="83" ht="42" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B83" s="12">
+    <row r="83" ht="42" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" s="12">
         <v>46150</v>
       </c>
-      <c r="C83" s="13" t="s">
+      <c r="B83" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D83" s="13" t="s">
+      <c r="C83" s="14" t="s">
         <v>135</v>
       </c>
+      <c r="D83" s="14">
+        <v>223.98</v>
+      </c>
       <c r="E83" s="14">
-        <v>223.98</v>
+        <v>0</v>
       </c>
       <c r="F83" s="14">
-        <v>0</v>
+        <v>15.68</v>
       </c>
       <c r="G83" s="14">
-        <v>15.68</v>
+        <v>0</v>
       </c>
       <c r="H83" s="15">
-        <v>0</v>
-      </c>
-      <c r="I83" s="16">
         <v>239.66</v>
       </c>
-      <c r="J83" s="4" t="s">
+      <c r="I83" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="K83">
+      <c r="J83" s="4">
         <v>2</v>
       </c>
     </row>
@@ -3666,19 +3668,19 @@
         <v>13</v>
       </c>
       <c r="D84" s="17">
-        <v>4759.67</v>
+        <v>4983.65</v>
       </c>
       <c r="E84" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F84" s="17">
-        <v>263.37</v>
+        <v>279.05</v>
       </c>
       <c r="G84" s="17">
         <v>3227.24</v>
       </c>
       <c r="H84" s="17">
-        <v>5243.41</v>
+        <v>5483.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>